<commit_message>
Update sample data with full stock names
Added complete ETF/stock names to db/Home_IRP.xlsx:
- ROI sheet: All 11 stocks now have Korean names
- Portfolio sheet: All 11 stocks now have Korean names

Examples:
- 449170: TIGER KOFR금리액티브(합성)
- 411060: ACE KRX금현물
- 379800: KODEX 미국S&P500
- 379810: KODEX 미국나스닥100
- etc.

This provides a complete view of the portfolio when users first
open the application.
</commit_message>
<xml_diff>
--- a/db/Home_IRP.xlsx
+++ b/db/Home_IRP.xlsx
@@ -473,7 +473,11 @@
           <t>449170</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TIGER KOFR금리액티브(합성)</t>
+        </is>
+      </c>
       <c r="C2" t="n">
         <v>5504005</v>
       </c>
@@ -496,7 +500,11 @@
           <t>411060</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ACE KRX금현물</t>
+        </is>
+      </c>
       <c r="C3" t="n">
         <v>1942055</v>
       </c>
@@ -519,7 +527,11 @@
           <t>468630</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>KODEX iShares미국투자등급회사채액티브</t>
+        </is>
+      </c>
       <c r="C4" t="n">
         <v>736740</v>
       </c>
@@ -542,7 +554,11 @@
           <t>476760</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ACE 미국30년국채액티브</t>
+        </is>
+      </c>
       <c r="C5" t="n">
         <v>1291165</v>
       </c>
@@ -565,7 +581,11 @@
           <t>0046A0</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TIGER 미국초단기(3개월이하)국채</t>
+        </is>
+      </c>
       <c r="C6" t="n">
         <v>331495</v>
       </c>
@@ -588,7 +608,11 @@
           <t>273130</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>KODEX 종합채권(AA-이상)액티브</t>
+        </is>
+      </c>
       <c r="C7" t="n">
         <v>446440</v>
       </c>
@@ -611,7 +635,11 @@
           <t>379800</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>KODEX 미국S&amp;P500</t>
+        </is>
+      </c>
       <c r="C8" t="n">
         <v>1627410</v>
       </c>
@@ -634,7 +662,11 @@
           <t>379810</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>KODEX 미국나스닥100</t>
+        </is>
+      </c>
       <c r="C9" t="n">
         <v>1716035</v>
       </c>
@@ -657,7 +689,11 @@
           <t>489250</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>KODEX 미국배당다우존스</t>
+        </is>
+      </c>
       <c r="C10" t="n">
         <v>1990000</v>
       </c>
@@ -680,7 +716,11 @@
           <t>294400</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>KIWOOM 200TR</t>
+        </is>
+      </c>
       <c r="C11" t="n">
         <v>443243</v>
       </c>
@@ -703,7 +743,11 @@
           <t>453870</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TIGER 인도니프티50</t>
+        </is>
+      </c>
       <c r="C12" t="n">
         <v>912282</v>
       </c>
@@ -855,7 +899,11 @@
           <t>449170</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TIGER KOFR금리액티브(합성)</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>안전자산</t>
@@ -882,7 +930,11 @@
           <t>411060</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ACE KRX금현물</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>대체자산</t>
@@ -909,7 +961,11 @@
           <t>468630</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>KODEX iShares미국투자등급회사채액티브</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>채권</t>
@@ -936,7 +992,11 @@
           <t>476760</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ACE 미국30년국채액티브</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>채권</t>
@@ -963,7 +1023,11 @@
           <t>0046A0</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TIGER 미국초단기(3개월이하)국채</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>채권</t>
@@ -990,7 +1054,11 @@
           <t>273130</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>KODEX 종합채권(AA-이상)액티브</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>채권</t>
@@ -1017,7 +1085,11 @@
           <t>379800</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>KODEX 미국S&amp;P500</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>주식</t>
@@ -1044,7 +1116,11 @@
           <t>379810</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>KODEX 미국나스닥100</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>주식</t>
@@ -1071,7 +1147,11 @@
           <t>489250</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>KODEX 미국배당다우존스</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>주식</t>
@@ -1098,7 +1178,11 @@
           <t>294400</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>KIWOOM 200TR</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>주식</t>
@@ -1125,7 +1209,11 @@
           <t>453870</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TIGER 인도니프티50</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>주식</t>

</xml_diff>

<commit_message>
Restructure Balance table and add auto-fill feature
- Merge 연도 and 월 columns into single 날짜 column (YYYYMMDD format)
- Remove 기타 column
- Auto-fill new Balance rows with:
  - Date from selected DB file (data_XXXX_YYYYMMDD.xlsx)
  - Investment principal from ROI total
  - Balance from ROI evaluation total
  - Return rate from ROI total
- Update column widths for new structure
- Update database files with new Balance sheet structure
</commit_message>
<xml_diff>
--- a/db/Home_IRP.xlsx
+++ b/db/Home_IRP.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="ROI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Balance" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Portfolio" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Portfolio" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Balance" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -775,72 +775,386 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>연도</t>
+          <t>종목코드</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>월</t>
+          <t>종목명</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>투자원금</t>
+          <t>자산군</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>추가납입</t>
+          <t>구분</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>잔고</t>
+          <t>세팅비중</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>수익률</t>
+          <t>현재비중</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>기타</t>
+          <t>녹색매수</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025년</t>
+          <t>449170</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>11월</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>16940870</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
+          <t>TIGER KOFR금리액티브(합성)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>안전자산</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>현금</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>18360634</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>8.4%</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F2" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-3894961</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>411060</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ACE KRX금현물</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>대체자산</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>금</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F3" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="G3" t="n">
+        <v>443370</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>468630</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>KODEX iShares미국투자등급회사채액티브</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>미국회사채</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>127022</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>476760</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ACE 미국30년국채액티브</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>미국장기채</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-385623</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0046A0</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TIGER 미국초단기(3개월이하)국채</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>미국단기채</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G6" t="n">
+        <v>123076</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>273130</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>KODEX 종합채권(AA-이상)액티브</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>국채</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-6064</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>379800</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>KODEX 미국S&amp;P500</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>미국지수</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>20</v>
+      </c>
+      <c r="F8" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1951837</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>379810</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>KODEX 미국나스닥100</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>미국지수</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>20</v>
+      </c>
+      <c r="F9" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1523827</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>489250</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>KODEX 미국배당다우존스</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>미국배당</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="G10" t="n">
+        <v>47133</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>294400</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>KIWOOM 200TR</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>국내지수</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G11" t="n">
+        <v>196982</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>453870</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TIGER 인도니프티50</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>신흥국</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-126598</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -853,385 +1167,55 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>종목코드</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>종목명</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>자산군</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>구분</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>세팅비중</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>현재비중</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>녹색매수</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>날짜</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>투자원금</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>추가납입</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>잔고</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>수익률</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>449170</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>TIGER KOFR금리액티브(합성)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>안전자산</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>현금</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F2" t="n">
-        <v>31.2</v>
-      </c>
-      <c r="G2" t="n">
-        <v>-3894961</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>411060</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ACE KRX금현물</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>대체자산</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>금</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>15</v>
-      </c>
-      <c r="F3" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="G3" t="n">
-        <v>443370</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>468630</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>KODEX iShares미국투자등급회사채액티브</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>채권</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>미국회사채</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="G4" t="n">
-        <v>127022</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>476760</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ACE 미국30년국채액티브</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>채권</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>미국장기채</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F5" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>-385623</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>0046A0</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>TIGER 미국초단기(3개월이하)국채</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>채권</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>미국단기채</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="G6" t="n">
-        <v>123076</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>273130</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>KODEX 종합채권(AA-이상)액티브</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>채권</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>국채</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G7" t="n">
-        <v>-6064</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>379800</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>KODEX 미국S&amp;P500</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>주식</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>미국지수</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>20</v>
-      </c>
-      <c r="F8" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1951837</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>379810</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>KODEX 미국나스닥100</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>주식</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>미국지수</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>20</v>
-      </c>
-      <c r="F9" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1523827</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>489250</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>KODEX 미국배당다우존스</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>주식</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>미국배당</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>10</v>
-      </c>
-      <c r="F10" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="G10" t="n">
-        <v>47133</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>294400</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>KIWOOM 200TR</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>주식</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>국내지수</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>5</v>
-      </c>
-      <c r="F11" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="G11" t="n">
-        <v>196982</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>453870</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>TIGER 인도니프티50</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>주식</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>신흥국</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>5</v>
-      </c>
-      <c r="F12" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="G12" t="n">
-        <v>-126598</v>
+          <t>20251101</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>16940870</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>18360634</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>8.4%</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>